<commit_message>
Update binary file for SSDLC AI model analysis
</commit_message>
<xml_diff>
--- a/開發文件/WI-GA215-附件一、SSDLC檢核表_AI輔助系統(語音轉文字).xlsx
+++ b/開發文件/WI-GA215-附件一、SSDLC檢核表_AI輔助系統(語音轉文字).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Speech-to-text\開發文件\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11C3E3A-7702-427F-8C09-B3A3BE073B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79546344-8FC6-4057-86AF-8C9CB5EA75B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2325" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="2310" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="130">
   <si>
     <t>SSDLC檢核表</t>
   </si>
@@ -57,9 +57,6 @@
     <t>是否依據資通系統防護基準需求分級？</t>
   </si>
   <si>
-    <t>V</t>
-  </si>
-  <si>
     <t>本系統屬於中低風險應用，已評估數據敏感性並實施對應級別的安全控制</t>
   </si>
   <si>
@@ -189,9 +186,6 @@
     <t>是否建立足夠之安全連線機制，如TLS.1.2以上？</t>
   </si>
   <si>
-    <t>HSTS標頭強制HTTPS，支持TLS 1.2+，安全標頭（X-Content-Type-Options, X-Frame-Options, CSP等）</t>
-  </si>
-  <si>
     <t>3.開發與測試階段</t>
   </si>
   <si>
@@ -282,166 +276,173 @@
     <t>是否將測試與線上環境進行區隔？</t>
   </si>
   <si>
+    <t>4.3</t>
+  </si>
+  <si>
+    <t>是否將程式開發、系統上線人員、資料庫管理員及網管人員進行職責區隔？</t>
+  </si>
+  <si>
+    <t>4.4</t>
+  </si>
+  <si>
+    <t>是否制定系統上線計畫（包含上線前中後之安裝、測試、問題排除、網路申請等）及留存相關紀錄？</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>是否制定系統版本發佈與更新程序，並留存相關紀錄？</t>
+  </si>
+  <si>
+    <t>4.6</t>
+  </si>
+  <si>
+    <t>是否針對委託單位之相關人員，進行系統操作與安全教育訓練？</t>
+  </si>
+  <si>
+    <t>5.維運階段</t>
+  </si>
+  <si>
+    <t>5.1</t>
+  </si>
+  <si>
+    <t>是否根據各項變更之需求，重複上述3~4流程已確認變更作業程序，並留存相關紀錄？</t>
+  </si>
+  <si>
+    <t>5.2</t>
+  </si>
+  <si>
+    <t>進行上述變更作業，是否對既有系統備份，並留存相關紀錄？</t>
+  </si>
+  <si>
+    <t>5.3</t>
+  </si>
+  <si>
+    <t>5.4</t>
+  </si>
+  <si>
+    <t>是否定期依法將過期之資料刪除，並留下刪除之記路？如個資保存期限</t>
+  </si>
+  <si>
+    <t>任務數據：處理完成後立即刪除；臨時文件：自動清理；日誌：超過期限自動輪替刪除；所有刪除操作記錄在audit.log</t>
+  </si>
+  <si>
+    <t>6.1</t>
+  </si>
+  <si>
+    <t>是否依規定將資料備份或銷燬，並依據資料安全性等級保存於規定的環境，並留存相關記錄？</t>
+  </si>
+  <si>
+    <t>資料庫之採用是否具備遮罩、HASH或編碼等機制？</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使用記憶體存儲，無傳統資料庫，敏感數據使用加密或HASH</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每個用戶使用唯一郵箱地址，所有操作記錄來源IP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>採用郵箱+驗證碼雙因子認證機制</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>包含個人資料：郵箱地址，無財務數據</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日誌文件自動輪替和備份（保留180-1825天），任務完成後自動清理相關文件</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日誌寫入失敗會輸出警告</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有日誌使用系統時間</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>統一API入口，所有請求經過安全中介軟體，郵箱驗證端點需驗證碼，管理員端點需ADMIN_TOKEN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>已文件化。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>開發環境（localhost）、生產環境（獨立部署）通過環境變數區分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>已實施Bandit 靜態分析、pip-audit 依賴漏洞掃描。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>管理員Token存放於環境變數，不硬編碼，加密金鑰自動生成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>requirements.txt指定最新穩定版本</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使用Git進行版本管理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>可參考文件：部屬指南.md、維運手冊.md</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>提供完整文檔：README.md, 部屬指南.md、維運手冊.md、安全文件.md</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>代碼變更通過Git管理、配置變更記錄在文檔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>若為硬體擴充或虛擬化，是否重複上述3~4流程已確認變更作業程序，並留存相關紀錄？</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>非為為硬體擴充或虛擬化。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日誌：自動輪替備份，保存180-1825天，建議定期備份至外部存儲；數據銷毀：安全刪除機制（覆寫3次），刪除操作記錄在audit.log</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>有進行職責區隔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>此為內部系統，評估尚不需要HTTPS。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6.系統下線階段</t>
+  </si>
+  <si>
+    <t>□</t>
+  </si>
+  <si>
+    <t>■</t>
+  </si>
+  <si>
+    <t>■</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>配置文件(.env)備份、日誌文件定期備份、代碼使用Git版本控制</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>通過環境變數區分環境，不同環境使用不同的.env配置</t>
-  </si>
-  <si>
-    <t>4.3</t>
-  </si>
-  <si>
-    <t>是否將程式開發、系統上線人員、資料庫管理員及網管人員進行職責區隔？</t>
-  </si>
-  <si>
-    <t>4.4</t>
-  </si>
-  <si>
-    <t>是否制定系統上線計畫（包含上線前中後之安裝、測試、問題排除、網路申請等）及留存相關紀錄？</t>
-  </si>
-  <si>
-    <t>4.5</t>
-  </si>
-  <si>
-    <t>是否制定系統版本發佈與更新程序，並留存相關紀錄？</t>
-  </si>
-  <si>
-    <t>4.6</t>
-  </si>
-  <si>
-    <t>是否針對委託單位之相關人員，進行系統操作與安全教育訓練？</t>
-  </si>
-  <si>
-    <t>5.維運階段</t>
-  </si>
-  <si>
-    <t>5.1</t>
-  </si>
-  <si>
-    <t>是否根據各項變更之需求，重複上述3~4流程已確認變更作業程序，並留存相關紀錄？</t>
-  </si>
-  <si>
-    <t>5.2</t>
-  </si>
-  <si>
-    <t>進行上述變更作業，是否對既有系統備份，並留存相關紀錄？</t>
-  </si>
-  <si>
-    <t>5.3</t>
-  </si>
-  <si>
-    <t>5.4</t>
-  </si>
-  <si>
-    <t>是否定期依法將過期之資料刪除，並留下刪除之記路？如個資保存期限</t>
-  </si>
-  <si>
-    <t>任務數據：處理完成後立即刪除；臨時文件：自動清理；日誌：超過期限自動輪替刪除；所有刪除操作記錄在audit.log</t>
-  </si>
-  <si>
-    <t>6.1</t>
-  </si>
-  <si>
-    <t>是否依規定將資料備份或銷燬，並依據資料安全性等級保存於規定的環境，並留存相關記錄？</t>
-  </si>
-  <si>
-    <t>資料庫之採用是否具備遮罩、HASH或編碼等機制？</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用記憶體存儲，無傳統資料庫，敏感數據使用加密或HASH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>每個用戶使用唯一郵箱地址，所有操作記錄來源IP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>採用郵箱+驗證碼雙因子認證機制</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>包含個人資料：郵箱地址，無財務數據</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>日誌文件自動輪替和備份（保留180-1825天），任務完成後自動清理相關文件</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>日誌寫入失敗會輸出警告</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>所有日誌使用系統時間</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>統一API入口，所有請求經過安全中介軟體，郵箱驗證端點需驗證碼，管理員端點需ADMIN_TOKEN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>已文件化。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>開發環境（localhost）、生產環境（獨立部署）通過環境變數區分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>V</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>已實施Bandit 靜態分析、pip-audit 依賴漏洞掃描。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用HTTPS/TLS傳輸，HSTS標頭強制HTTPS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>管理員Token存放於環境變數，不硬編碼，加密金鑰自動生成</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>requirements.txt指定最新穩定版本</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>未進行職責區隔</t>
-  </si>
-  <si>
-    <t>未進行職責區隔</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用Git進行版本管理</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>可參考文件：部屬指南.md、維運手冊.md</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>提供完整文檔：README.md, 部屬指南.md、維運手冊.md、安全文件.md</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>代碼變更通過Git管理、配置變更記錄在文檔</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>配置文件(.env)備份、日誌文件定期備份、代碼使用Git版本控制</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>若為硬體擴充或虛擬化，是否重複上述3~4流程已確認變更作業程序，並留存相關紀錄？</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>非為為硬體擴充或虛擬化。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>日誌：自動輪替備份，保存180-1825天，建議定期備份至外部存儲；數據銷毀：安全刪除機制（覆寫3次），刪除操作記錄在audit.log</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -629,7 +630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -660,6 +661,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -670,11 +677,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -980,6 +989,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F53"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -987,19 +999,19 @@
     <col min="2" max="2" width="47.375" style="1" customWidth="1"/>
     <col min="3" max="4" width="7.125" style="11" customWidth="1"/>
     <col min="5" max="5" width="8.125" style="11" customWidth="1"/>
-    <col min="6" max="6" width="88.625" style="19" customWidth="1"/>
+    <col min="6" max="6" width="88.625" style="13" customWidth="1"/>
     <col min="7" max="7" width="14.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -1017,19 +1029,19 @@
       <c r="E2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="14"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="16"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -1038,13 +1050,17 @@
       <c r="B4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>9</v>
-      </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="8" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1052,15 +1068,19 @@
         <v>1.2</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>11</v>
-      </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="8" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1068,15 +1088,19 @@
         <v>1.3</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="8" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1084,15 +1108,19 @@
         <v>1.4</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>15</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="8" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1100,15 +1128,19 @@
         <v>1.5</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F8" s="8" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1116,15 +1148,19 @@
         <v>1.6</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F9" s="8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1132,15 +1168,19 @@
         <v>1.7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F10" s="8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1148,15 +1188,19 @@
         <v>1.8</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>20</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="8" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1164,57 +1208,69 @@
         <v>1.9</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="8" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="8" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="14"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>2.1</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>27</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="8" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1222,15 +1278,19 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>29</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1238,15 +1298,19 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>31</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="8" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1254,15 +1318,19 @@
         <v>2.4</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="8" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1270,15 +1338,19 @@
         <v>2.5</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1286,15 +1358,19 @@
         <v>2.6</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1302,15 +1378,19 @@
         <v>2.7</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F21" s="8" t="s">
         <v>39</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="8" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1318,15 +1398,19 @@
         <v>2.8</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F22" s="8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1334,482 +1418,593 @@
         <v>2.9</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F23" s="8" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F24" s="8" t="s">
         <v>44</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="8" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="8" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="C26" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F26" s="8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E27" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="14"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="16"/>
     </row>
     <row r="29" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E29" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F29" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="8" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E30" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F30" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F31" s="8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="E32" s="10"/>
+        <v>61</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F32" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F33" s="8" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F34" s="8" t="s">
         <v>66</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="8" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F35" s="8" t="s">
         <v>69</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D36" s="10"/>
+        <v>71</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D36" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="E36" s="10" t="s">
-        <v>9</v>
+        <v>126</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
+        <v>101</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D37" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="E37" s="10" t="s">
-        <v>9</v>
+        <v>126</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
+        <v>74</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F38" s="8" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D39" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E39" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="14"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="16"/>
     </row>
     <row r="41" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D41" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E41" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F41" s="8" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D42" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E42" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F42" s="8" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
+      </c>
+      <c r="C43" s="23" t="s">
+        <v>125</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E43" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="E43" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F43" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D44" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E44" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F44" s="8" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D45" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E45" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F45" s="8" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D46" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E46" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F46" s="8" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="14"/>
+      <c r="A47" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="16"/>
     </row>
     <row r="48" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D48" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E48" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F48" s="8" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D49" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E49" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F49" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C50" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50" s="10"/>
+        <v>119</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D50" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="E50" s="10" t="s">
-        <v>9</v>
+        <v>126</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D51" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E51" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F51" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="12"/>
-      <c r="B52" s="13"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="14"/>
+      <c r="A52" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B52" s="20"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="22"/>
     </row>
     <row r="53" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
+        <v>126</v>
+      </c>
+      <c r="D53" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E53" s="23" t="s">
+        <v>125</v>
+      </c>
       <c r="F53" s="8" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A52:F52"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A52:F52"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293"/>
+  <pageSetup paperSize="9" scale="58" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>